<commit_message>
Harden MCDM methods and add Monte Carlo UI
</commit_message>
<xml_diff>
--- a/AURA_MonteCarlo_Results.xlsx
+++ b/AURA_MonteCarlo_Results.xlsx
@@ -480,10 +480,10 @@
         <v>3</v>
       </c>
       <c r="C2" t="n">
-        <v>3.7592</v>
+        <v>3.7272</v>
       </c>
       <c r="D2" t="n">
-        <v>2.394789209930595</v>
+        <v>2.359360116641798</v>
       </c>
       <c r="E2" t="n">
         <v>1</v>
@@ -492,7 +492,7 @@
         <v>11</v>
       </c>
       <c r="G2" t="n">
-        <v>77.79000000000001</v>
+        <v>78.39</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -508,10 +508,10 @@
         <v>1</v>
       </c>
       <c r="C3" t="n">
-        <v>3.9288</v>
+        <v>3.9678</v>
       </c>
       <c r="D3" t="n">
-        <v>3.560664342506887</v>
+        <v>3.597716381261869</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -520,10 +520,10 @@
         <v>13</v>
       </c>
       <c r="G3" t="n">
-        <v>75.79000000000001</v>
+        <v>75.88000000000001</v>
       </c>
       <c r="H3" t="n">
-        <v>3.11</v>
+        <v>3.64</v>
       </c>
     </row>
     <row r="4">
@@ -536,10 +536,10 @@
         <v>4</v>
       </c>
       <c r="C4" t="n">
-        <v>4.2111</v>
+        <v>4.1961</v>
       </c>
       <c r="D4" t="n">
-        <v>1.490079457612915</v>
+        <v>1.505936515926219</v>
       </c>
       <c r="E4" t="n">
         <v>1</v>
@@ -548,7 +548,7 @@
         <v>8</v>
       </c>
       <c r="G4" t="n">
-        <v>80.02</v>
+        <v>80.11</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -564,10 +564,10 @@
         <v>6</v>
       </c>
       <c r="C5" t="n">
-        <v>5.399</v>
+        <v>5.444</v>
       </c>
       <c r="D5" t="n">
-        <v>3.486488061072345</v>
+        <v>3.533166285359352</v>
       </c>
       <c r="E5" t="n">
         <v>1</v>
@@ -576,7 +576,7 @@
         <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>50.73999999999999</v>
+        <v>50.82</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -592,10 +592,10 @@
         <v>2</v>
       </c>
       <c r="C6" t="n">
-        <v>5.4617</v>
+        <v>5.4838</v>
       </c>
       <c r="D6" t="n">
-        <v>3.696015842769076</v>
+        <v>3.690736723203106</v>
       </c>
       <c r="E6" t="n">
         <v>1</v>
@@ -604,10 +604,10 @@
         <v>13</v>
       </c>
       <c r="G6" t="n">
-        <v>62.74999999999999</v>
+        <v>62.3</v>
       </c>
       <c r="H6" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="7">
@@ -620,10 +620,10 @@
         <v>8</v>
       </c>
       <c r="C7" t="n">
-        <v>5.5918</v>
+        <v>5.5612</v>
       </c>
       <c r="D7" t="n">
-        <v>2.569274753699962</v>
+        <v>2.578537290791041</v>
       </c>
       <c r="E7" t="n">
         <v>1</v>
@@ -632,7 +632,7 @@
         <v>10</v>
       </c>
       <c r="G7" t="n">
-        <v>41.68</v>
+        <v>41.88</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -648,10 +648,10 @@
         <v>5</v>
       </c>
       <c r="C8" t="n">
-        <v>6.5676</v>
+        <v>6.5704</v>
       </c>
       <c r="D8" t="n">
-        <v>1.6496151793676</v>
+        <v>1.635189236755184</v>
       </c>
       <c r="E8" t="n">
         <v>3</v>
@@ -660,7 +660,7 @@
         <v>11</v>
       </c>
       <c r="G8" t="n">
-        <v>28.65</v>
+        <v>28.2</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -676,10 +676,10 @@
         <v>9</v>
       </c>
       <c r="C9" t="n">
-        <v>6.9344</v>
+        <v>6.9327</v>
       </c>
       <c r="D9" t="n">
-        <v>2.821187097659423</v>
+        <v>2.806202186229638</v>
       </c>
       <c r="E9" t="n">
         <v>1</v>
@@ -688,7 +688,7 @@
         <v>12</v>
       </c>
       <c r="G9" t="n">
-        <v>35.5</v>
+        <v>35.78</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -704,10 +704,10 @@
         <v>7</v>
       </c>
       <c r="C10" t="n">
-        <v>8.2614</v>
+        <v>8.3055</v>
       </c>
       <c r="D10" t="n">
-        <v>4.679516004887685</v>
+        <v>4.701592256884895</v>
       </c>
       <c r="E10" t="n">
         <v>1</v>
@@ -716,10 +716,10 @@
         <v>15</v>
       </c>
       <c r="G10" t="n">
-        <v>34.11</v>
+        <v>33.7</v>
       </c>
       <c r="H10" t="n">
-        <v>28.81</v>
+        <v>29.46</v>
       </c>
     </row>
     <row r="11">
@@ -732,10 +732,10 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>8.3765</v>
+        <v>8.3773</v>
       </c>
       <c r="D11" t="n">
-        <v>1.455660588873656</v>
+        <v>1.455796932954593</v>
       </c>
       <c r="E11" t="n">
         <v>4</v>
@@ -744,7 +744,7 @@
         <v>11</v>
       </c>
       <c r="G11" t="n">
-        <v>4.3</v>
+        <v>4.34</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -760,10 +760,10 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>9.6958</v>
+        <v>9.6754</v>
       </c>
       <c r="D12" t="n">
-        <v>2.479770626489474</v>
+        <v>2.474234192634157</v>
       </c>
       <c r="E12" t="n">
         <v>3</v>
@@ -772,10 +772,10 @@
         <v>14</v>
       </c>
       <c r="G12" t="n">
-        <v>7.79</v>
+        <v>7.69</v>
       </c>
       <c r="H12" t="n">
-        <v>7.68</v>
+        <v>7.779999999999999</v>
       </c>
     </row>
     <row r="13">
@@ -788,10 +788,10 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>11.0567</v>
+        <v>11.045</v>
       </c>
       <c r="D13" t="n">
-        <v>1.630179471714694</v>
+        <v>1.652868718319758</v>
       </c>
       <c r="E13" t="n">
         <v>4</v>
@@ -800,10 +800,10 @@
         <v>13</v>
       </c>
       <c r="G13" t="n">
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
       <c r="H13" t="n">
-        <v>10.11</v>
+        <v>9.59</v>
       </c>
     </row>
     <row r="14">
@@ -816,10 +816,10 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>12.0097</v>
+        <v>11.9902</v>
       </c>
       <c r="D14" t="n">
-        <v>1.277186716968197</v>
+        <v>1.29880866951218</v>
       </c>
       <c r="E14" t="n">
         <v>8</v>
@@ -831,7 +831,7 @@
         <v>0</v>
       </c>
       <c r="H14" t="n">
-        <v>53.54</v>
+        <v>53.19</v>
       </c>
     </row>
     <row r="15">
@@ -844,10 +844,10 @@
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>13.8968</v>
+        <v>13.8798</v>
       </c>
       <c r="D15" t="n">
-        <v>0.5971178778097337</v>
+        <v>0.6159155461587246</v>
       </c>
       <c r="E15" t="n">
         <v>12</v>
@@ -859,7 +859,7 @@
         <v>0</v>
       </c>
       <c r="H15" t="n">
-        <v>96.89</v>
+        <v>96.38</v>
       </c>
     </row>
     <row r="16">
@@ -872,10 +872,10 @@
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>14.8495</v>
+        <v>14.8436</v>
       </c>
       <c r="D16" t="n">
-        <v>0.3909600363208496</v>
+        <v>0.3897935864018288</v>
       </c>
       <c r="E16" t="n">
         <v>12</v>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="H16" t="n">
-        <v>99.70999999999999</v>
+        <v>99.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>